<commit_message>
donnees: regenerer l'annexe 1 et les exports — grille a 28, 24 certifies, 19 instrumentes, unites alignees (M3, S4), serie A2 et avances T5/T6
</commit_message>
<xml_diff>
--- a/exports/1_tableau_de_veille.xlsx
+++ b/exports/1_tableau_de_veille.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>10.08.2026 à 09:42</t>
+          <t>12.08.2026 à 22:18</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="K4" s="11" t="n">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="O4" s="11" t="n">
-        <v>351</v>
+        <v>378</v>
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="Q4" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="K7" s="11" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="P7" s="11" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="Q7" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -1857,13 +1857,17 @@
           <t>https://www.acea.auto</t>
         </is>
       </c>
-      <c r="O9" s="12" t="inlineStr">
-        <is>
-          <t>aucune collecte</t>
-        </is>
-      </c>
-      <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="11" t="n"/>
+      <c r="O9" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P9" s="11" t="inlineStr">
+        <is>
+          <t>2025-11 → 2025-11</t>
+        </is>
+      </c>
+      <c r="Q9" s="11" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -1994,7 +1998,7 @@
         </is>
       </c>
       <c r="K11" s="11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
@@ -2012,7 +2016,7 @@
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
@@ -2020,7 +2024,7 @@
         </is>
       </c>
       <c r="Q11" s="11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -2075,7 +2079,7 @@
         </is>
       </c>
       <c r="K12" s="11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
@@ -2093,7 +2097,7 @@
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>656</v>
+        <v>697</v>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
@@ -2101,7 +2105,7 @@
         </is>
       </c>
       <c r="Q12" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -2156,7 +2160,7 @@
         </is>
       </c>
       <c r="K13" s="11" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="L13" s="11" t="inlineStr">
         <is>
@@ -2174,15 +2178,15 @@
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>99</v>
+        <v>550</v>
       </c>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>2024-01 → 2024-03</t>
+          <t>2023-01 → 2026-05</t>
         </is>
       </c>
       <c r="Q13" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -2314,7 +2318,7 @@
         </is>
       </c>
       <c r="K15" s="11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
@@ -2332,7 +2336,7 @@
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="P15" s="11" t="inlineStr">
         <is>
@@ -2340,7 +2344,7 @@
         </is>
       </c>
       <c r="Q15" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -2547,7 +2551,7 @@
         </is>
       </c>
       <c r="K18" s="11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
@@ -2565,7 +2569,7 @@
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="P18" s="11" t="inlineStr">
         <is>
@@ -2573,7 +2577,7 @@
         </is>
       </c>
       <c r="Q18" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -2628,7 +2632,7 @@
         </is>
       </c>
       <c r="K19" s="11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="L19" s="11" t="inlineStr">
         <is>
@@ -2646,7 +2650,7 @@
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="P19" s="11" t="inlineStr">
         <is>
@@ -2654,7 +2658,7 @@
         </is>
       </c>
       <c r="Q19" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -3015,7 +3019,7 @@
         </is>
       </c>
       <c r="K24" s="11" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="L24" s="11" t="inlineStr">
         <is>
@@ -3033,7 +3037,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="P24" s="11" t="inlineStr">
         <is>
@@ -3041,7 +3045,7 @@
         </is>
       </c>
       <c r="Q24" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -3096,7 +3100,7 @@
         </is>
       </c>
       <c r="K25" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
@@ -3114,7 +3118,7 @@
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>1032</v>
+        <v>1118</v>
       </c>
       <c r="P25" s="11" t="inlineStr">
         <is>
@@ -3122,7 +3126,7 @@
         </is>
       </c>
       <c r="Q25" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26">
@@ -3270,7 +3274,7 @@
         </is>
       </c>
       <c r="O27" s="11" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P27" s="11" t="inlineStr">
         <is>
@@ -3278,7 +3282,7 @@
         </is>
       </c>
       <c r="Q27" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prototype: passe de preuve avant assemblage — liste du figeage soldée, part du document A1 mesurée à 1 %, socle et exports régénérés
Deux harnais verts. Trois écarts texte/base corrigés côté rapport (215
exécutions, M6 = 20, part A1 ≈ 1 % mesurée dans les exécutions n8n 1803-1806
au lieu de 2,5 %). Migration corrigeant la note de source d'A1 ; générateurs
des annexes 2 et 4 alignés ; db/ régénéré et rejoué en recette ; annexe 1 et
classeur régénérés ; fichiers bruts du run 214 archivés hors dépôt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VhAt6L5jFS2YcZA2j9AxnN
</commit_message>
<xml_diff>
--- a/exports/1_tableau_de_veille.xlsx
+++ b/exports/1_tableau_de_veille.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Couverture QV'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lacunes'!$A$1:$H$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Lacunes'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$1:$L$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Sources'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -632,7 +632,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>02.09.2026 à 07:55</t>
+          <t>04.09.2026 à 18:33</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Statistiques de production automobile</t>
+          <t>Production mondiale de véhicules par pays — tableau republié dans l'annuaire du CCFA « L'industrie automobile française » (mention imprimée « Source : OICA »), document collecté ; classements top-10 de la page OICA en vérité terrain</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="M11" s="11" t="inlineStr">
         <is>
-          <t>Tableaux web</t>
+          <t>PDF (annuaire CCFA, https://ccfa.fr/analyses-et-statistiques/) ; tableaux web OICA pour la confrontation opportuniste</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr">
@@ -7250,10 +7250,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -7392,77 +7392,77 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>aie</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>Global EV Data Explorer</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>Agence internationale de l'énergie</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>acea_incitations</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Electric cars: tax benefits and incentives (fiscalité et aides à l'achat, par pays)</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>ACEA</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>annuelle</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>CSV</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>PDF tabulaire (tableau comparatif par pays)</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>certifiee</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>07.08.2026</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
-        <is>
-          <t>A11, A3</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>https://www.iea.org</t>
-        </is>
-      </c>
-      <c r="L3" s="11" t="n"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>02.09.2026</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="n"/>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>https://www.acea.auto/fact/electric-cars-tax-benefits-and-incentives-2025/</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Issue de la couche 0 (run du 22.08.2026, QV5 automobile, candidat 2, 3 modèles sur 4). Inscrite le 02.09.2026 sans liaison de collecte : accès vérifié en réponse réelle (HTTP 200 les 22.08 et 02.09), granularité d'extraction non validée. Pas d'indicateur rattaché à ce jour.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>banque_mondiale</t>
+          <t>aie</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Séries macroéconomiques mondiales</t>
+          <t>Global EV Data Explorer</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Banque mondiale</t>
+          <t>Agence internationale de l'énergie</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>API + CSV</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
@@ -7495,10 +7495,14 @@
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J4" s="11" t="n"/>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>A11, A3</t>
+        </is>
+      </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>https://data.worldbank.org</t>
+          <t>https://www.iea.org</t>
         </is>
       </c>
       <c r="L4" s="11" t="n"/>
@@ -7506,27 +7510,27 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>bns</t>
+          <t>banque_mondiale</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Taux de change de référence</t>
+          <t>Séries macroéconomiques mondiales</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Banque nationale suisse</t>
+          <t>Banque mondiale</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>mensuelle</t>
+          <t>annuelle</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>API / CSV</t>
+          <t>API + CSV</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -7549,14 +7553,10 @@
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
+      <c r="J5" s="11" t="n"/>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>https://data.snb.ch</t>
+          <t>https://data.worldbank.org</t>
         </is>
       </c>
       <c r="L5" s="11" t="n"/>
@@ -7564,32 +7564,32 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>comtrade</t>
+          <t>bns</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>UN Comtrade : commerce international par code SH</t>
+          <t>Taux de change de référence</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Nations Unies</t>
+          <t>Banque nationale suisse</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>annuelle</t>
+          <t>mensuelle</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>API + CSV</t>
+          <t>API / CSV</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>libre_quota</t>
+          <t>libre</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -7609,49 +7609,45 @@
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>A4, H1, H3, M1, S6</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>https://comtradeplus.un.org</t>
-        </is>
-      </c>
-      <c r="L6" s="11" t="inlineStr">
-        <is>
-          <t>Quota sur l'API publique</t>
-        </is>
-      </c>
+          <t>https://data.snb.ch</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>constructeurs</t>
+          <t>comtrade</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Commandes et livraisons d'avions commerciaux</t>
+          <t>UN Comtrade : commerce international par code SH</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Airbus, Boeing</t>
+          <t>Nations Unies</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>mensuelle</t>
+          <t>annuelle</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Web / Excel</t>
+          <t>API + CSV</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>libre_quota</t>
         </is>
       </c>
       <c r="G7" s="11" t="inlineStr">
@@ -7671,44 +7667,44 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>A4, H1, H3, M1, S6</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
+          <t>https://comtradeplus.un.org</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>Deux producteurs à consolider</t>
+          <t>Quota sur l'API publique</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>cp</t>
+          <t>constructeurs</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Recensement du personnel et des entreprises des industries horlogère et microtechnique suisses</t>
+          <t>Commandes et livraisons d'avions commerciaux</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Convention patronale de l'industrie horlogère suisse</t>
+          <t>Airbus, Boeing</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>annuelle</t>
+          <t>mensuelle</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>PDF (lecture multimodale)</t>
+          <t>Web / Excel</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
@@ -7728,287 +7724,287 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>30.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>H11, H2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>https://cpih.ch/statistiques/</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Association patronale, PAS une statistique publique — provenance à déclarer comme pour la FH (§ 8.6.4) ; ne jamais étiqueter « donnée officielle ». Recensement au 30 septembre, publication en décembre. La page d'index est STABLE, le nom du PDF change chaque année : le lien se résout depuis l'index, comme pour la FH et le classeur SIPRI. Tableau Tb. 1e = série 2005-2025, effectifs et entreprises.</t>
+          <t>Deux producteurs à consolider</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
+          <t>cp</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Recensement du personnel et des entreprises des industries horlogère et microtechnique suisses</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Convention patronale de l'industrie horlogère suisse</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>annuelle</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>PDF (lecture multimodale)</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>certifiee</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>N. Castillo</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>30.08.2026</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>H11, H2</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>https://cpih.ch/statistiques/</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>Association patronale, PAS une statistique publique — provenance à déclarer comme pour la FH (§ 8.6.4) ; ne jamais étiqueter « donnée officielle ». Recensement au 30 septembre, publication en décembre. La page d'index est STABLE, le nom du PDF change chaque année : le lien se résout depuis l'index, comme pour la FH et le classeur SIPRI. Tableau Tb. 1e = série 2005-2025, effectifs et entreprises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
           <t>cpb</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>World Trade Monitor</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>CPB Netherlands Bureau for Economic Policy Analysis</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>mensuelle</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>certifiee</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="K9" s="11" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>https://www.cpb.nl/en/worldtrademonitor/latest</t>
         </is>
       </c>
-      <c r="L9" s="11" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>URL corrigée le 24.08.2026 : l'ancienne (…/en/worldtrademonitor) renvoyait 404. La nouvelle redirige vers le millésime courant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>deloitte</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Swiss Watch Industry Study</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Deloitte</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>annuelle</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>libre</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>a_confirmer</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>N. Castillo</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>07.08.2026</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>H5</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>https://www.deloitte.com/ch</t>
-        </is>
-      </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>Étude annuelle, méthodologie déclarative</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
+          <t>deloitte</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Swiss Watch Industry Study</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>annuelle</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>N. Castillo</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>07.08.2026</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>https://www.deloitte.com/ch</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>Étude annuelle, méthodologie déclarative</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
           <t>esa</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Budgets spatiaux publics</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>ESA et agences nationales</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>annuelle</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>a_confirmer</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="I12" s="13" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J12" s="13" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
       </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="K12" s="13" t="inlineStr">
         <is>
           <t>https://www.esa.int</t>
         </is>
       </c>
-      <c r="L11" s="13" t="inlineStr">
+      <c r="L12" s="13" t="inlineStr">
         <is>
           <t>Formats hétérogènes selon les agences</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>eurostat</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Eurostat : statistiques conjoncturelles et structurelles</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Commission européenne</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>mensuelle</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>API + CSV</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>libre</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>certifiee</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>N. Castillo</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>07.08.2026</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>A5, A6, H6, M2, S8, T10, T11, T5, T7, T8, T9</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>https://ec.europa.eu/eurostat/data/database</t>
-        </is>
-      </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>API de dissémination sans authentification</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>fh</t>
+          <t>eurostat</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Statistiques d'exportation horlogère</t>
+          <t>Eurostat : statistiques conjoncturelles et structurelles</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Fédération de l'industrie horlogère suisse</t>
+          <t>Commission européenne</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -8018,7 +8014,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>PDF / communiqués</t>
+          <t>API + CSV</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -8038,221 +8034,221 @@
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>09.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>H7, H8, H9</t>
+          <t>A5, A6, H6, M2, S8, T10, T11, T5, T7, T8, T9</t>
         </is>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>https://www.fhs.swiss</t>
+          <t>https://ec.europa.eu/eurostat/data/database</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>Détail par marché de destination. Provenance précisée le 27.08.2026 : la FH rediffuse la statistique douanière suisse du commerce extérieur (OFDF) en y ajoutant le détail de branche (mécanique/quartz, destinations) — source secondaire d'un chiffre officiel, qualifiée comme référence de branche.</t>
+          <t>API de dissémination sans authentification</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
+          <t>fh</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Statistiques d'exportation horlogère</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Fédération de l'industrie horlogère suisse</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>mensuelle</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>PDF / communiqués</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>certifiee</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>N. Castillo</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>09.08.2026</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>H7, H8, H9</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>https://www.fhs.swiss</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Détail par marché de destination. Provenance précisée le 27.08.2026 : la FH rediffuse la statistique douanière suisse du commerce extérieur (OFDF) en y ajoutant le détail de branche (mécanique/quartz, destinations) — source secondaire d'un chiffre officiel, qualifiée comme référence de branche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
           <t>fmi</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>World Economic Outlook</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Fonds monétaire international</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>semestrielle</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>CSV</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>certifiee</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="K14" s="11" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>https://www.imf.org/en/Publications/WEO</t>
         </is>
       </c>
-      <c r="L14" s="11" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="L15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>iata</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Air Passenger Market Analysis</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>IATA</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>mensuelle</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>a_confirmer</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I16" s="13" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="K15" s="13" t="inlineStr">
+      <c r="K16" s="13" t="inlineStr">
         <is>
           <t>https://www.iata.org</t>
         </is>
       </c>
-      <c r="L15" s="13" t="inlineStr">
+      <c r="L16" s="13" t="inlineStr">
         <is>
           <t>Séries détaillées réservées aux membres</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>kof</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Baromètre conjoncturel KOF</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>KOF ETH Zurich</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>mensuelle</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>API / CSV</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>libre</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>certifiee</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>N. Castillo</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>17.08.2026</t>
-        </is>
-      </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>https://data.kof.ethz.ch</t>
-        </is>
-      </c>
-      <c r="L16" s="11" t="inlineStr">
-        <is>
-          <t>API v2 publique sans clé (access_type=public), CSV date/valeur, mensuel depuis 1991. Vérifiée en réponse réelle le 17.08.2026. Ancienne API v1 hors service — motif du re-sourçage documenté.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>ocde</t>
+          <t>kof</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Principaux indicateurs économiques et CLI</t>
+          <t>Baromètre conjoncturel KOF</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>OCDE</t>
+          <t>KOF ETH Zurich</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -8262,7 +8258,7 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>API + CSV</t>
+          <t>API / CSV</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -8282,34 +8278,34 @@
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>07.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T6</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>https://data-explorer.oecd.org</t>
+          <t>https://data.kof.ethz.ch</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>Vérifié le 10.08.2026 : la série CLI est vivante et mensuelle, mais l'agrégat « OCDE total » n'est plus publié — 22 zones disponibles dont G20, G7, G4E, NAFTA. T1 réancré sur G20. Version du flux non épinglée : la 4.1 ne porte plus la mesure LI. Limitation de débit annoncée par la documentation sans être chiffrée.</t>
+          <t>API v2 publique sans clé (access_type=public), CSV date/valeur, mensuel depuis 1991. Vérifiée en réponse réelle le 17.08.2026. Ancienne API v1 hors service — motif du re-sourçage documenté.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>ocde_brevets</t>
+          <t>ocde</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Brevets par domaine technologique</t>
+          <t>Principaux indicateurs économiques et CLI</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -8319,12 +8315,12 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>annuelle</t>
+          <t>mensuelle</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>API SDMX</t>
+          <t>API + CSV</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -8344,39 +8340,39 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>25.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>A7, M6</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>https://data-explorer.oecd.org/vis?df[ag]=OECD.STI.PIE&amp;df[id]=DSD_PATENTS@DF_PATENTS_OECDSPECIFIC</t>
+          <t>https://data-explorer.oecd.org</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>Jeu DF_PATENTS_OECDSPECIFIC. Dix-huit domaines technologiques, dont MEDICAL et TRA (technologies de transport bas carbone). Sans clé. Vérifié en réponse réelle le 25.08.2026 : 13 points annuels 2010-2022, 106 zones disponibles.</t>
+          <t>Vérifié le 10.08.2026 : la série CLI est vivante et mensuelle, mais l'agrégat « OCDE total » n'est plus publié — 22 zones disponibles dont G20, G7, G4E, NAFTA. T1 réancré sur G20. Version du flux non épinglée : la 4.1 ne porte plus la mesure LI. Limitation de débit annoncée par la documentation sans être chiffrée.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>ofs</t>
+          <t>ocde_brevets</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>STATENT : Etablissements et emplois selon année, canton, genre économique et unité d'observation (table px-x-0602010000_103)</t>
+          <t>Brevets par domaine technologique</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Office fédéral de la statistique</t>
+          <t>OCDE</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -8386,7 +8382,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>API PX-Web (JSON-stat2, requête POST)</t>
+          <t>API SDMX</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -8406,39 +8402,39 @@
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>30.08.2026</t>
+          <t>25.08.2026</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>H12, M4</t>
+          <t>A7, M6</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>https://www.pxweb.bfs.admin.ch/api/v1/fr/px-x-0602010000_103/px-x-0602010000_103.px</t>
+          <t>https://data-explorer.oecd.org/vis?df[ag]=OECD.STI.PIE&amp;df[id]=DSD_PATENTS@DF_PATENTS_OECDSPECIFIC</t>
         </is>
       </c>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>Nomenclature NOGA. Cube STATENT interrogé en POST : le seul URL ne rend pas la donnée, le corps de requête fait partie de la référence (voir source_bindings 142 et 143). H2 = cinq classes NOGA 2652 sommées ; M4 = NOGA 266000 et 3250xx. Unité d'observation 2 (emplois) ; la modalité 1 (établissements) est identifiée, non instrumentée. Consultation à l'écran de la même table : https://www.pxweb.bfs.admin.ch/pxweb/fr/px-x-0602010000_103/px-x-0602010000_103/px-x-0602010000_103.px</t>
+          <t>Jeu DF_PATENTS_OECDSPECIFIC. Dix-huit domaines technologiques, dont MEDICAL et TRA (technologies de transport bas carbone). Sans clé. Vérifié en réponse réelle le 25.08.2026 : 13 points annuels 2010-2022, 106 zones disponibles.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>oica</t>
+          <t>ofs</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Statistiques de production automobile</t>
+          <t>STATENT : Etablissements et emplois selon année, canton, genre économique et unité d'observation (table px-x-0602010000_103)</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>OICA</t>
+          <t>Office fédéral de la statistique</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -8448,7 +8444,7 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Tableaux web</t>
+          <t>API PX-Web (JSON-stat2, requête POST)</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
@@ -8468,35 +8464,39 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>07.08.2026</t>
+          <t>30.08.2026</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>H12, M4</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>https://www.oica.net/production-statistics</t>
-        </is>
-      </c>
-      <c r="L20" s="11" t="n"/>
+          <t>https://www.pxweb.bfs.admin.ch/api/v1/fr/px-x-0602010000_103/px-x-0602010000_103.px</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>Nomenclature NOGA. Cube STATENT interrogé en POST : le seul URL ne rend pas la donnée, le corps de requête fait partie de la référence (voir source_bindings 142 et 143). H2 = cinq classes NOGA 2652 sommées ; M4 = NOGA 266000 et 3250xx. Unité d'observation 2 (emplois) ; la modalité 1 (établissements) est identifiée, non instrumentée. Consultation à l'écran de la même table : https://www.pxweb.bfs.admin.ch/pxweb/fr/px-x-0602010000_103/px-x-0602010000_103/px-x-0602010000_103.px</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>ompi</t>
+          <t>oica</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Statistiques de propriété intellectuelle</t>
+          <t>Production mondiale de véhicules par pays — tableau republié dans l'annuaire du CCFA « L'industrie automobile française » (mention imprimée « Source : OICA »), document collecté ; classements top-10 de la page OICA en vérité terrain</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>OMPI</t>
+          <t>OICA</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>PDF (annuaire CCFA, https://ccfa.fr/analyses-et-statistiques/) ; tableaux web OICA pour la confrontation opportuniste</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -8526,34 +8526,34 @@
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>07.08.2026</t>
+          <t>31.08.2026</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/ipstats</t>
+          <t>https://www.oica.net/production-statistics</t>
         </is>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>Classification CIB</t>
+          <t>Producteur : OICA. Document collecté : annuaire CCFA (association professionnelle française), PDF, une édition par an, tableau « La production mondiale de véhicules » par pays en milliers, mention « Source : OICA » imprimée. Éditions traitées au 31.08.2026 : page des analyses et statistiques (édition courante), CCFA-2023, CCFA-2024 (composite_queue 9-11), série 2021-2024. Découpe par sentinelles avant envoi aux modèles (~1 % du document : 5 100 caractères sur ~530 000, mesuré sur les exécutions du 31.08.2026 ; corrigé de 2,5 % le 04.09). Vérité terrain de rang 1 : classements top-10 de https://www.oica.net/production-statistics, JSON incorporé, confrontation opportuniste (non_verifiable quand l'année n'est pas servie, jamais de faux verdict). Détection des nouvelles éditions : workflow veille_documentaire_annuelle.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>ompi_tech</t>
+          <t>ompi</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Indicateurs de brevets par domaine technologique</t>
+          <t>Statistiques de propriété intellectuelle</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>ZIP / CSV</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -8588,39 +8588,39 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>25.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>T12, T13</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/en/web/ip-statistics</t>
+          <t>https://www.wipo.int/ipstats</t>
         </is>
       </c>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>Archive wipo-data-patent-indicators.zip, téléchargement direct sans inscription. Comptages par année, office, pays d'origine et domaine technologique (35 domaines). Vérifié en réponse réelle le 25.08.2026 : 663 584 lignes, 2000-2022. Table de concordance CIB/domaine publiée séparément et consultée pour établir les limites de granularité — G04 tombe dans « Techniques de mesure », B64 dans « Transport ».</t>
+          <t>Classification CIB</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>oms_ghed</t>
+          <t>ompi_tech</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Global Health Expenditure Database</t>
+          <t>Indicateurs de brevets par domaine technologique</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>OMS</t>
+          <t>OMPI</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>API / CSV</t>
+          <t>ZIP / CSV</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
@@ -8650,45 +8650,49 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>07.08.2026</t>
+          <t>25.08.2026</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>T12, T13</t>
         </is>
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>https://apps.who.int/nha/database</t>
-        </is>
-      </c>
-      <c r="L23" s="11" t="n"/>
+          <t>https://www.wipo.int/en/web/ip-statistics</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>Archive wipo-data-patent-indicators.zip, téléchargement direct sans inscription. Comptages par année, office, pays d'origine et domaine technologique (35 domaines). Vérifié en réponse réelle le 25.08.2026 : 663 584 lignes, 2000-2022. Table de concordance CIB/domaine publiée séparément et consultée pour établir les limites de granularité — G04 tombe dans « Techniques de mesure », B64 dans « Transport ».</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>openfda</t>
+          <t>oms_ghed</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>openFDA : bases publiques de la Food and Drug Administration</t>
+          <t>Global Health Expenditure Database</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>U.S. Food and Drug Administration</t>
+          <t>OMS</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>quotidienne</t>
+          <t>annuelle</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>API / CSV</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
@@ -8708,333 +8712,391 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>https://open.fda.gov</t>
-        </is>
-      </c>
-      <c r="L24" s="11" t="inlineStr">
-        <is>
-          <t>API libre et sans clé (quota anonyme). Vérifiée en réponse réelle le 23.08.2026 : onze mois consécutifs de décomptes 510(k). Deux pièges d'appel consignés — la syntaxe d'intervalle « champ:[debut+TO+fin] » ne doit pas voir son « + » encodé (sinon 500), et une recherche sans résultat répond 404 et non 200 avec liste vide.</t>
-        </is>
-      </c>
+          <t>https://apps.who.int/nha/database</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
+          <t>openfda</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>openFDA : bases publiques de la Food and Drug Administration</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>U.S. Food and Drug Administration</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>quotidienne</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>certifiee</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>N. Castillo</t>
+        </is>
+      </c>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>https://open.fda.gov</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>API libre et sans clé (quota anonyme). Vérifiée en réponse réelle le 23.08.2026 : onze mois consécutifs de décomptes 510(k). Deux pièges d'appel consignés — la syntaxe d'intervalle « champ:[debut+TO+fin] » ne doit pas voir son « + » encodé (sinon 500), et une recherche sans résultat répond 404 et non 200 avec liste vide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
           <t>sipri</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Military Expenditure Database</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>SIPRI</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>annuelle</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>CSV</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>certifiee</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>https://www.sipri.org/databases/milex</t>
         </is>
       </c>
-      <c r="L25" s="11" t="inlineStr">
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>URL corrigée le 24.08.2026 : l'ancienne (milex.sipri.org) échouait à la négociation TLS. Adresse alignée sur celle de la liaison S4.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>swiss_medtech</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Swiss Medical Technology Industry report</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Swiss Medtech</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>bisannuelle</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E27" s="13" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="G27" s="13" t="inlineStr">
         <is>
           <t>a_confirmer</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H27" s="13" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="K26" s="13" t="inlineStr">
+      <c r="K27" s="13" t="inlineStr">
         <is>
           <t>https://www.swiss-medtech.ch</t>
         </is>
       </c>
-      <c r="L26" s="13" t="inlineStr">
+      <c r="L27" s="13" t="inlineStr">
         <is>
           <t>Publication bisannuelle, périodes non alignées sur la fenêtre 2023-2025</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>ted</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Tenders Electronic Daily : marchés publics UE</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Office des publications de l'UE</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>quotidienne</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>API</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>certifiee</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>20.08.2026</t>
         </is>
       </c>
-      <c r="J27" s="11" t="inlineStr">
+      <c r="J28" s="11" t="inlineStr">
         <is>
           <t>A8, M7, S7</t>
         </is>
       </c>
-      <c r="K27" s="11" t="inlineStr">
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>https://ted.europa.eu</t>
         </is>
       </c>
-      <c r="L27" s="11" t="inlineStr">
+      <c r="L28" s="11" t="inlineStr">
         <is>
           <t>API de recherche v3, POST JSON, sans clé pour la recherche. Vérifiée en réponse réelle le 20.08.2026 (totalNoticeCount par requête CPV + bornes de dates). Source de la famille OSINT F3 (marchés publics) de la demande de ratification.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>triage_flux</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Intensité de signalement dans les flux qualifiés (dérivation interne)</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>Dispositif de veille : dérivation du triage IA (v_intensite_signalement)</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>mensuelle</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>sql</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G28" s="13" t="inlineStr">
+      <c r="G29" s="13" t="inlineStr">
         <is>
           <t>a_confirmer</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="H29" s="13" t="inlineStr">
         <is>
           <t>N. Castillo (délégation du 27.08.2026)</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="I29" s="13" t="inlineStr">
         <is>
           <t>27.08.2026</t>
         </is>
       </c>
-      <c r="J28" s="13" t="inlineStr">
+      <c r="J29" s="13" t="inlineStr">
         <is>
           <t>A10, A9, H10, S9</t>
         </is>
       </c>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K29" s="13" t="inlineStr">
         <is>
           <t>interne : flux_sources → flux_items → flux_triage_ia → v_intensite_signalement</t>
         </is>
       </c>
-      <c r="L28" s="13" t="inlineStr">
+      <c r="L29" s="13" t="inlineStr">
         <is>
           <t>Non pas une source externe mais une dérivation : part mensuelle des items triés attribués à une question de veille. Hérite de la qualification des flux sous-jacents (tous en accès libre). a_confirmer tant que le corpus est jeune (démarré fin 07.2026) et sa composition mouvante.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>unoosa</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Objets lancés dans l'espace</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>UNOOSA / Our World in Data</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>annuelle</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>CSV</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>libre</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>certifiee</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>N. Castillo</t>
         </is>
       </c>
-      <c r="I29" s="11" t="inlineStr">
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J29" s="11" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="K29" s="11" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>https://ourworldindata.org/space-exploration-satellites</t>
         </is>
       </c>
-      <c r="L29" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:L30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>